<commit_message>
feat(currency-wars): implement activity runtime
</commit_message>
<xml_diff>
--- a/config/currency-wars-generated/templates/CurrencyWars.xlsx
+++ b/config/currency-wars-generated/templates/CurrencyWars.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6035" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6085" uniqueCount="313">
   <si>
     <t>@table</t>
   </si>
@@ -327,7 +327,7 @@
     <t>CurrencyWarsNodes</t>
   </si>
   <si>
-    <t>fcc06569aa366c25</t>
+    <t>f02b0ac0cd2b5082</t>
   </si>
   <si>
     <t>layer_id</t>
@@ -342,6 +342,27 @@
     <t>room_pool_id</t>
   </si>
   <si>
+    <t>node_template_id</t>
+  </si>
+  <si>
+    <t>stage_id</t>
+  </si>
+  <si>
+    <t>node_type</t>
+  </si>
+  <si>
+    <t>parameter_ids</t>
+  </si>
+  <si>
+    <t>penalty_bonus_rule_id</t>
+  </si>
+  <si>
+    <t>basic_gold_reward</t>
+  </si>
+  <si>
+    <t>next_node_id</t>
+  </si>
+  <si>
     <t>CurrencyWarsDomainCompositions</t>
   </si>
   <si>
@@ -447,7 +468,7 @@
     <t>CurrencyWarsRosterAvatars</t>
   </si>
   <si>
-    <t>102876bc4cbb195f</t>
+    <t>77a3f7bb812b702a</t>
   </si>
   <si>
     <t>avatar_id</t>
@@ -456,12 +477,18 @@
     <t>cost</t>
   </si>
   <si>
+    <t>rarity</t>
+  </si>
+  <si>
     <t>role_id</t>
   </si>
   <si>
     <t>build_mapping_id</t>
   </si>
   <si>
+    <t>position_kind</t>
+  </si>
+  <si>
     <t>CurrencyWarsEconomyRules</t>
   </si>
   <si>
@@ -516,7 +543,7 @@
     <t>CurrencyWarsTeamSizeStates</t>
   </si>
   <si>
-    <t>83b2449ce83507fc</t>
+    <t>1b663b531aeb7279</t>
   </si>
   <si>
     <t>level</t>
@@ -528,6 +555,9 @@
     <t>bench_cap</t>
   </si>
   <si>
+    <t>next_level_experience</t>
+  </si>
+  <si>
     <t>CurrencyWarsRoleMappings</t>
   </si>
   <si>
@@ -544,9 +574,6 @@
   </si>
   <si>
     <t>97aa01b869b05be9</t>
-  </si>
-  <si>
-    <t>position_kind</t>
   </si>
   <si>
     <t>field_index</t>
@@ -2129,7 +2156,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:Z7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2143,10 +2170,13 @@
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
     <col min="15" max="17" width="16.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="21.7109375" style="5" customWidth="1"/>
-    <col min="19" max="19" width="16.7109375" style="5" customWidth="1"/>
+    <col min="19" max="23" width="16.7109375" style="5" customWidth="1"/>
+    <col min="24" max="24" width="21.7109375" style="5" customWidth="1"/>
+    <col min="25" max="25" width="17.7109375" style="5" customWidth="1"/>
+    <col min="26" max="26" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2178,7 +2208,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="24" customHeight="1">
+    <row r="2" spans="1:26" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -2236,8 +2266,29 @@
       <c r="S2" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="3" spans="1:19">
+      <c r="T2" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26">
       <c r="A3" s="4" t="s">
         <v>28</v>
       </c>
@@ -2295,8 +2346,29 @@
       <c r="S3" s="5" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="4" spans="1:19">
+      <c r="T3" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26">
       <c r="A4" s="4" t="s">
         <v>29</v>
       </c>
@@ -2354,8 +2426,29 @@
       <c r="S4" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:19">
+      <c r="T4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26">
       <c r="A5" s="4" t="s">
         <v>33</v>
       </c>
@@ -2413,8 +2506,29 @@
       <c r="S5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:19">
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26">
       <c r="A6" s="4" t="s">
         <v>34</v>
       </c>
@@ -2472,8 +2586,29 @@
       <c r="S6" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" ht="42" customHeight="1">
+      <c r="T6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
@@ -2495,6 +2630,13 @@
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
       <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2531,7 +2673,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2555,7 +2697,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -2602,16 +2744,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>60</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -2658,16 +2800,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>60</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -2895,7 +3037,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2919,7 +3061,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -2966,16 +3108,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -3022,16 +3164,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -3257,7 +3399,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3281,7 +3423,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -3328,19 +3470,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -3387,19 +3529,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -3635,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3659,7 +3801,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -3706,16 +3848,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -3762,16 +3904,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -4000,7 +4142,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4024,7 +4166,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -4071,16 +4213,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -4127,16 +4269,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -4364,7 +4506,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4388,7 +4530,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -4435,10 +4577,10 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>56</v>
@@ -4488,10 +4630,10 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>56</v>
@@ -4690,7 +4832,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -4702,15 +4844,15 @@
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="18" width="16.7109375" style="5" customWidth="1"/>
+    <col min="15" max="20" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4734,10 +4876,10 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="24" customHeight="1">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -4781,19 +4923,25 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
+        <v>135</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
       <c r="A3" s="4" t="s">
         <v>28</v>
       </c>
@@ -4837,19 +4985,25 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18">
+        <v>135</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
       <c r="A4" s="4" t="s">
         <v>29</v>
       </c>
@@ -4904,8 +5058,14 @@
       <c r="R4" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:18">
+      <c r="S4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
       <c r="A5" s="4" t="s">
         <v>33</v>
       </c>
@@ -4960,8 +5120,14 @@
       <c r="R5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:18">
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
       <c r="A6" s="4" t="s">
         <v>34</v>
       </c>
@@ -5016,8 +5182,14 @@
       <c r="R6" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="S6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="T6" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
@@ -5038,6 +5210,8 @@
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -5072,7 +5246,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5096,7 +5270,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -5143,16 +5317,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -5199,16 +5373,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -5798,7 +5972,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5822,7 +5996,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -5869,16 +6043,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -5925,16 +6099,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -6161,7 +6335,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6185,7 +6359,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -6232,16 +6406,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -6288,16 +6462,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -6503,7 +6677,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -6515,15 +6689,17 @@
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="18" width="16.7109375" style="5" customWidth="1"/>
+    <col min="15" max="17" width="16.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="21.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6547,10 +6723,10 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="24" customHeight="1">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -6594,19 +6770,22 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="R2" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="S2" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:19">
       <c r="A3" s="4" t="s">
         <v>28</v>
       </c>
@@ -6650,19 +6829,22 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="R3" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="S3" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:19">
       <c r="A4" s="4" t="s">
         <v>29</v>
       </c>
@@ -6717,8 +6899,11 @@
       <c r="R4" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:18">
+      <c r="S4" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
       <c r="A5" s="4" t="s">
         <v>33</v>
       </c>
@@ -6773,8 +6958,11 @@
       <c r="R5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:18">
+      <c r="S5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
       <c r="A6" s="4" t="s">
         <v>34</v>
       </c>
@@ -6829,8 +7017,11 @@
       <c r="R6" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="42" customHeight="1">
+      <c r="S6" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
@@ -6851,6 +7042,7 @@
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -6885,7 +7077,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6909,7 +7101,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -6956,13 +7148,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -7009,13 +7201,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -7232,7 +7424,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7256,7 +7448,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -7303,16 +7495,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -7359,16 +7551,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -7594,7 +7786,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7618,7 +7810,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -7665,19 +7857,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -7724,19 +7916,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -7974,7 +8166,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7998,7 +8190,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -8045,19 +8237,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>55</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -8104,19 +8296,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -8352,7 +8544,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8376,7 +8568,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -8423,16 +8615,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -8479,16 +8671,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -8714,7 +8906,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8738,7 +8930,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -8785,16 +8977,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -8841,16 +9033,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -9076,7 +9268,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9100,7 +9292,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -9147,19 +9339,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -9206,19 +9398,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -9816,7 +10008,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9840,7 +10032,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -9887,16 +10079,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -9943,16 +10135,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -10178,7 +10370,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10202,7 +10394,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -10249,16 +10441,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -10305,16 +10497,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -10540,7 +10732,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10564,7 +10756,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -10611,16 +10803,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -10667,16 +10859,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -10902,7 +11094,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10926,7 +11118,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -10973,16 +11165,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -11029,16 +11221,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -11264,7 +11456,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -11288,7 +11480,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -11335,16 +11527,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -11391,16 +11583,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -11626,7 +11818,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -11650,7 +11842,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -11697,19 +11889,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -11756,19 +11948,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -12006,7 +12198,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -12030,7 +12222,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -12077,16 +12269,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -12133,16 +12325,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -12369,7 +12561,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -12393,7 +12585,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -12440,16 +12632,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -12496,16 +12688,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -12731,7 +12923,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -12755,7 +12947,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -12802,16 +12994,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -12858,16 +13050,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -13093,7 +13285,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -13117,7 +13309,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -13164,22 +13356,22 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -13226,22 +13418,22 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -13849,7 +14041,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -13873,7 +14065,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -13920,19 +14112,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>55</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -13979,19 +14171,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -14227,7 +14419,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -14251,7 +14443,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -14298,13 +14490,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>55</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -14351,13 +14543,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -14573,7 +14765,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -14597,7 +14789,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="24" customHeight="1">
@@ -14644,10 +14836,10 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -14694,10 +14886,10 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -14903,7 +15095,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -14927,7 +15119,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -14974,16 +15166,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>55</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -15030,16 +15222,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -15265,7 +15457,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -15289,7 +15481,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -15339,10 +15531,10 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -15392,10 +15584,10 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -15611,7 +15803,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -15635,7 +15827,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -15682,13 +15874,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -15735,13 +15927,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -15957,7 +16149,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -15981,7 +16173,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="24" customHeight="1">
@@ -16028,10 +16220,10 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -16078,10 +16270,10 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -16287,7 +16479,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -16311,7 +16503,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -16358,16 +16550,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -16414,16 +16606,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -16649,7 +16841,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -16673,7 +16865,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -16720,19 +16912,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>55</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -16779,19 +16971,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -17027,7 +17219,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -17051,7 +17243,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="24" customHeight="1">
@@ -17098,10 +17290,10 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -17148,10 +17340,10 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -17704,7 +17896,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -17728,7 +17920,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -17775,19 +17967,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>55</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -17834,19 +18026,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -18082,7 +18274,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -18106,7 +18298,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -18153,16 +18345,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -18209,16 +18401,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -18444,7 +18636,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -18468,7 +18660,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="24" customHeight="1">
@@ -18515,10 +18707,10 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -18565,10 +18757,10 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -18774,7 +18966,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -18798,7 +18990,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="24" customHeight="1">
@@ -18845,10 +19037,10 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -18895,10 +19087,10 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>277</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -19104,7 +19296,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -19128,7 +19320,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -19175,22 +19367,22 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -19237,22 +19429,22 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -19498,7 +19690,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -19522,7 +19714,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -19569,16 +19761,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>55</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -19625,16 +19817,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -19860,7 +20052,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -19884,7 +20076,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -19931,19 +20123,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -19990,19 +20182,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -20238,7 +20430,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -20262,7 +20454,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -20309,19 +20501,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>55</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -20368,19 +20560,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>55</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -20616,7 +20808,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -20640,7 +20832,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -20687,16 +20879,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -20743,16 +20935,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -20979,7 +21171,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -21003,7 +21195,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -21056,7 +21248,7 @@
         <v>65</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -21109,7 +21301,7 @@
         <v>65</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -21672,7 +21864,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -21696,7 +21888,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -21743,16 +21935,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -21799,16 +21991,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
     </row>
     <row r="4" spans="1:18">

</xml_diff>